<commit_message>
added formatting for landlordRate and added mhiyMarginVal
</commit_message>
<xml_diff>
--- a/scripts/Excel Files/bookings_formatted.xlsx
+++ b/scripts/Excel Files/bookings_formatted.xlsx
@@ -6447,7 +6447,7 @@
         <v>1923309</v>
       </c>
       <c r="C46" t="str">
-        <v>Ethan Mavuzi</v>
+        <v>Orla Dunne</v>
       </c>
       <c r="D46" t="str">
         <v>Orla Dunne</v>
@@ -8847,7 +8847,7 @@
         <v>1920591</v>
       </c>
       <c r="C64" t="str">
-        <v>Ethan Mavuzi</v>
+        <v>Orla Dunne</v>
       </c>
       <c r="D64" t="str">
         <v>Orla Dunne</v>
@@ -49651,7 +49651,7 @@
         <v>1923511-EXT-3</v>
       </c>
       <c r="C369" t="str">
-        <v>Orla Dunne</v>
+        <v>Ornela Zalli</v>
       </c>
       <c r="D369" t="str">
         <v>Ornela Zalli</v>
@@ -51929,7 +51929,7 @@
         <v>1930901</v>
       </c>
       <c r="C386" t="str">
-        <v>Ethan Mavuzi</v>
+        <v>Luke Naumovi</v>
       </c>
       <c r="D386" t="str">
         <v>Luke Naumovi</v>

</xml_diff>